<commit_message>
Submission added to the journal
</commit_message>
<xml_diff>
--- a/docs/journal/IoT-Workshop_Journal_Gruppe4.xlsx
+++ b/docs/journal/IoT-Workshop_Journal_Gruppe4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a00eac15ea2058d9/Dokumente/Projektarbeit IoT/GreenHouse_Überarbeitet/Neues Project 2026/IoT-Workshop/docs/journal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{2CD16CF0-FEEF-46E2-A555-23F0981B504E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D7EDA24-C604-4964-ABD5-52706551D9DB}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{2CD16CF0-FEEF-46E2-A555-23F0981B504E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EE8E73B-0F0F-4636-A1C7-CED009A3883E}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{E915CADC-ACED-43ED-BD6F-EA5F35FC2958}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="109">
   <si>
     <t>Tag</t>
   </si>
@@ -357,6 +357,12 @@
   </si>
   <si>
     <t>IoT Workshop Gruppe 4 (Joël Rohner, Tobias Kulow)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abgabe Branch erstelllt </t>
+  </si>
+  <si>
+    <t>Vollständige Abgabe</t>
   </si>
 </sst>
 </file>
@@ -781,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{589255D4-02C3-423C-98CA-9E93BB57D3FC}">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="17.69140625" bestFit="1" customWidth="1"/>
@@ -1466,6 +1472,26 @@
         <v>105</v>
       </c>
     </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A32" s="3">
+        <v>46094</v>
+      </c>
+      <c r="B32" s="2">
+        <v>1</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G3"/>

</xml_diff>